<commit_message>
chore(testing): tester package and manifest for test build v0.13.0-rc.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMjJ2LeCjs6pJ2deXkbdAT
</commit_message>
<xml_diff>
--- a/testing/nyarlathotep-dev-round-01-production-setups.xlsx
+++ b/testing/nyarlathotep-dev-round-01-production-setups.xlsx
@@ -610,14 +610,14 @@
     <row r="2" ht="19" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Build: test build 0.13.0-rc.1 (apocalypse and unit watch, before release). Prepared 2026-10-14.</t>
+          <t>Build: test build 0.13.0-rc.2 (apocalypse, unit watch, faction wave templates and the fresh-world fix, before release). Prepared 2026-10-16.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="19" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Download: https://github.com/KDavidP1987/Nyarlathotep-Lord-of-Chaos/releases/tag/v0.13.0-rc.1</t>
+          <t>Download: https://github.com/KDavidP1987/Nyarlathotep-Lord-of-Chaos/releases/tag/v0.13.0-rc.2</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>1. Open the download page (link above) and download Nyarlathotep-0.13.0-rc.1.zip, this workbook and its reading copy -&gt; the zip holds Nyarlathotep.dll and a short install note.</t>
+          <t>1. Open the download page (link above) and download Nyarlathotep-0.13.0-rc.2.zip, this workbook and its reading copy -&gt; the zip holds Nyarlathotep.dll and a short install note.</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>6. Start the server and open BepInEx/LogOutput.log -&gt; a line 'Plugin kdpen.Nyarlathotep v0.13.0-rc.1 loaded' appears, and BepInEx/config gains kdpen.Nyarlathotep.cfg.</t>
+          <t>6. Start the server and open BepInEx/LogOutput.log -&gt; a line 'Plugin kdpen.Nyarlathotep v0.13.0-rc.2 loaded' appears, and BepInEx/config gains kdpen.Nyarlathotep.cfg.</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>8. In game, type .nyar in chat -&gt; the first line reads 'Nyarlathotep, Lord of Chaos (v0.13.0-rc.1)' and the admin commands are listed. Everything ships switched off; each row turns on what it needs.</t>
+          <t>8. In game, type .nyar in chat -&gt; the first line reads 'Nyarlathotep, Lord of Chaos (v0.13.0-rc.2)' and the admin commands are listed. Everything ships switched off; each row turns on what it needs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(testing): tester package and manifest for test build v0.13.0-rc.3
Rows N-18 (militia-muster-timed) and N-19 (undead-onslaught with pursuit);
download and install steps point at the rc.3 pre-release.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMjJ2LeCjs6pJ2deXkbdAT
</commit_message>
<xml_diff>
--- a/testing/nyarlathotep-dev-round-01-production-setups.xlsx
+++ b/testing/nyarlathotep-dev-round-01-production-setups.xlsx
@@ -16,8 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test plan'!$A$1:$P$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test steps'!$A$1:$F$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test plan'!$A$1:$P$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test steps'!$A$1:$F$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -610,14 +610,14 @@
     <row r="2" ht="19" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Build: test build 0.13.0-rc.2 (apocalypse, unit watch, faction wave templates and the fresh-world fix, before release). Prepared 2026-10-16.</t>
+          <t>Build: test build 0.13.0-rc.3 (apocalypse, unit watch, faction wave templates, pursuit and the timed and onslaught waves, before release). Prepared 2026-10-16.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="19" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Download: https://github.com/KDavidP1987/Nyarlathotep-Lord-of-Chaos/releases/tag/v0.13.0-rc.2</t>
+          <t>Download: https://github.com/KDavidP1987/Nyarlathotep-Lord-of-Chaos/releases/tag/v0.13.0-rc.3</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>1. Open the download page (link above) and download Nyarlathotep-0.13.0-rc.2.zip, this workbook and its reading copy -&gt; the zip holds Nyarlathotep.dll and a short install note.</t>
+          <t>1. Open the download page (link above) and download Nyarlathotep-0.13.0-rc.3.zip, this workbook and its reading copy -&gt; the zip holds Nyarlathotep.dll and a short install note.</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>6. Start the server and open BepInEx/LogOutput.log -&gt; a line 'Plugin kdpen.Nyarlathotep v0.13.0-rc.2 loaded' appears, and BepInEx/config gains kdpen.Nyarlathotep.cfg.</t>
+          <t>6. Start the server and open BepInEx/LogOutput.log -&gt; a line 'Plugin kdpen.Nyarlathotep v0.13.0-rc.3 loaded' appears, and BepInEx/config gains kdpen.Nyarlathotep.cfg.</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>8. In game, type .nyar in chat -&gt; the first line reads 'Nyarlathotep, Lord of Chaos (v0.13.0-rc.2)' and the admin commands are listed. Everything ships switched off; each row turns on what it needs.</t>
+          <t>8. In game, type .nyar in chat -&gt; the first line reads 'Nyarlathotep, Lord of Chaos (v0.13.0-rc.3)' and the admin commands are listed. Everything ships switched off; each row turns on what it needs.</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
     <row r="40" ht="49" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Connect to the dev server, the test server set up with the steps under 'Installing the build', at the address its admin gives you (Direct Connect, not the server list). 18 of the 20 rows need admin rights: the owner adds you as an admin before the round, and you type '.nyar' in chat to confirm you see the admin commands. Rows that need admin say so under 'You will need'.</t>
+          <t>Connect to the dev server, the test server set up with the steps under 'Installing the build', at the address its admin gives you (Direct Connect, not the server list). 20 of the 22 rows need admin rights: the owner adds you as an admin before the round, and you type '.nyar' in chat to confirm you see the admin commands. Rows that need admin say so under 'You will need'.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1836,111 +1836,175 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="21" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="20" ht="109" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>N-18</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Spawn events</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Timed waves: the next wave comes whether you are ready or not</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>New — this did not exist on the server before.</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>'Militia muster (timed)' is militia-muster on a clock: 5 waves of militia in a 40 m arena, a new wave every 75 seconds even if the last one is still alive, ending on the militia leader. Six other factions have a timed version too (names ending in -timed).</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Type .nyar template use militia-muster-timed, .nyar event enable militia-muster-timed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="124" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>N-19</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Spawn events</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Onslaught: random waves, surprise bosses, and no running away</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>New — this did not exist on the server before.</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>'Undead onslaught' rolls each wave at random from groups of undead, adds a random undead V Blood in the middle wave and one or two at the end. If nobody stays in the 40 m arena for 60 seconds, the undead go after the nearest player anywhere on the map. Six other factions have one too (names ending in -onslaught).</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Type .nyar template use undead-onslaught, .nyar event enable undead-onslaught, then .nyar event start undead-onslaught in open ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="21" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Established feature — a fresh pair of eyes</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="64" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
+    <row r="23" ht="64" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>E-01</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Spawn events</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>Build your own event from chat, the way a new admin would</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Not new; never looked at by a person.</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Without the documentation, create a new spawn event from scratch with chat commands, set it up as you would for your own server, and run it.</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>Type .nyar event new my-event spawns</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="64" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
+    <row r="24" ht="64" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>E-02</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Two players</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>A second player joins someone else's fight</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Not new; never looked at by a person.</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Take any event from the rows above that hunts one player (revenge, the border watch) and have a second player join in from the side.</t>
         </is>
       </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>Player one triggers N-08 or N-13</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="21" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+    <row r="25" ht="21" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Not an ordinary test row</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="79" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="26" ht="79" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>C-01</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Server feel</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Measurement: how the server feels during the busiest event</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>A measurement, not a change.</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>Not a pass or fail row. During the apocalypse (N-14), note any lag, rubber-banding or slow abilities, and when it happened. One reading is a baseline, not a series.</t>
         </is>
       </c>
-      <c r="F24" s="15" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>At the start, at each horde rise and at the end, note how responsive the game feels (fine, slight lag, bad lag) and the time.</t>
         </is>
@@ -1948,9 +2012,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A20:F20"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2186,7 +2250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3173,15 +3237,15 @@
       <c r="O18" s="17" t="n"/>
       <c r="P18" s="17" t="n"/>
     </row>
-    <row r="19" ht="34" customHeight="1">
+    <row r="19" ht="79" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>N-18</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>Established feature — a fresh pair of eyes</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
@@ -3191,12 +3255,12 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Build your own event from chat, the way a new admin would</t>
+          <t>Timed waves: the next wave comes whether you are ready or not</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>Admin rights; 20 minutes.</t>
+          <t>Admin rights; the Spawns kind on (.nyar pillar spawns on); two players with gear level 50 or more (the militia leader is level 58); open ground.</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
@@ -3204,7 +3268,7 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>Which reply or field name stopped you?</t>
+          <t>Did the pressure of the clock feel exciting or simply unfair?</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr">
@@ -3225,38 +3289,38 @@
       <c r="O19" s="17" t="n"/>
       <c r="P19" s="17" t="n"/>
     </row>
-    <row r="20" ht="34" customHeight="1">
+    <row r="20" ht="79" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>N-19</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Established feature — a fresh pair of eyes</t>
+          <t>New</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>Two players</t>
+          <t>Spawn events</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>A second player joins someone else's fight</t>
+          <t>Onslaught: random waves, surprise bosses, and no running away</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Two players at the same time.</t>
+          <t>Admin rights; the Spawns kind on; two players with gear level 60 or more (the undead V Bloods run from level 27 to 63, up to two at once); a castle nearby.</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>Did the fight still make sense with a second player in it?</t>
+          <t>Did the chase feel like a threat, and did anything visibly teleport while you watched?</t>
         </is>
       </c>
       <c r="H20" s="17" t="inlineStr">
@@ -3277,38 +3341,38 @@
       <c r="O20" s="17" t="n"/>
       <c r="P20" s="17" t="n"/>
     </row>
-    <row r="21" ht="49" customHeight="1">
+    <row r="21" ht="34" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>C-01</t>
+          <t>E-01</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Not an ordinary test row</t>
+          <t>Established feature — a fresh pair of eyes</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Server feel</t>
+          <t>Spawn events</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Measurement: how the server feels during the busiest event</t>
+          <t>Build your own event from chat, the way a new admin would</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>Being in the apocalypse run of N-14.</t>
+          <t>Admin rights; 20 minutes.</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>Was there any moment the server felt slower than usual, and when?</t>
+          <t>Which reply or field name stopped you?</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
@@ -3329,9 +3393,113 @@
       <c r="O21" s="17" t="n"/>
       <c r="P21" s="17" t="n"/>
     </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>E-02</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Established feature — a fresh pair of eyes</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Two players</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>A second player joins someone else's fight</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Two players at the same time.</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Did the fight still make sense with a second player in it?</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Not assigned yet</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>Not tested yet</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="n"/>
+      <c r="K22" s="17" t="n"/>
+      <c r="L22" s="17" t="n"/>
+      <c r="M22" s="17" t="n"/>
+      <c r="N22" s="17" t="n"/>
+      <c r="O22" s="17" t="n"/>
+      <c r="P22" s="17" t="n"/>
+    </row>
+    <row r="23" ht="49" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>C-01</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Not an ordinary test row</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Server feel</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Measurement: how the server feels during the busiest event</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Being in the apocalypse run of N-14.</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Was there any moment the server felt slower than usual, and when?</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Not assigned yet</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>Not tested yet</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="n"/>
+      <c r="K23" s="17" t="n"/>
+      <c r="L23" s="17" t="n"/>
+      <c r="M23" s="17" t="n"/>
+      <c r="N23" s="17" t="n"/>
+      <c r="O23" s="17" t="n"/>
+      <c r="P23" s="17" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P21"/>
-  <conditionalFormatting sqref="I2:I21">
+  <autoFilter ref="A1:P23"/>
+  <conditionalFormatting sqref="I2:I23">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>I2="Pass"</formula>
     </cfRule>
@@ -3349,10 +3517,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tester A,Tester B,Both — coordinated,Not assigned yet"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Partial pass,Fail,Blocked,Not tested yet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3367,7 +3535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5162,14 +5330,14 @@
     <row r="96" ht="21" customHeight="1">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>E-01 — Build your own event from chat, the way a new admin would</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="19" customHeight="1">
+          <t>N-18 — Timed waves: the next wave comes whether you are ready or not</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="34" customHeight="1">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>N-18</t>
         </is>
       </c>
       <c r="B97" s="15" t="n">
@@ -5177,21 +5345,17 @@
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event new my-event spawns</t>
-        </is>
-      </c>
-      <c r="D97" s="15" t="inlineStr">
-        <is>
-          <t>a switched-off event is created.</t>
-        </is>
-      </c>
+          <t>Type .nyar template use militia-muster-timed, .nyar event enable militia-muster-timed.</t>
+        </is>
+      </c>
+      <c r="D97" s="15" t="inlineStr"/>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="7" t="n"/>
     </row>
-    <row r="98" ht="49" customHeight="1">
+    <row r="98" ht="34" customHeight="1">
       <c r="A98" s="15" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>N-18</t>
         </is>
       </c>
       <c r="B98" s="15" t="n">
@@ -5199,17 +5363,21 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Use .nyar event set my-event ... to choose units (action.units, e.g. CHAR_Forest_Wolf:4), waves, the location (location here) and a level (action.modifiers.level 30).</t>
-        </is>
-      </c>
-      <c r="D98" s="15" t="inlineStr"/>
+          <t>Stand in open ground and type .nyar event start militia-muster-timed</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>wave 1 (6 militia) appears around you.</t>
+        </is>
+      </c>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="7" t="n"/>
     </row>
-    <row r="99" ht="19" customHeight="1">
+    <row r="99" ht="34" customHeight="1">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>N-18</t>
         </is>
       </c>
       <c r="B99" s="15" t="n">
@@ -5217,21 +5385,21 @@
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event info my-event, then enable and start it</t>
+          <t>Do not fight for a while</t>
         </is>
       </c>
       <c r="D99" s="15" t="inlineStr">
         <is>
-          <t>it runs as you set it.</t>
+          <t>about 75 seconds after the start, wave 2 (9 militia) arrives while wave 1 is still alive.</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="7" t="n"/>
     </row>
-    <row r="100" ht="19" customHeight="1">
+    <row r="100" ht="49" customHeight="1">
       <c r="A100" s="15" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>N-18</t>
         </is>
       </c>
       <c r="B100" s="15" t="n">
@@ -5239,24 +5407,28 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Note every reply that confused you, word for word.</t>
-        </is>
-      </c>
-      <c r="D100" s="15" t="inlineStr"/>
+          <t>Fight the rest</t>
+        </is>
+      </c>
+      <c r="D100" s="15" t="inlineStr">
+        <is>
+          <t>waves keep coming every 75 seconds; wave 5 brings the militia leader; the scoreboard names a winner at the end.</t>
+        </is>
+      </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="7" t="n"/>
     </row>
     <row r="101" ht="21" customHeight="1">
       <c r="A101" s="18" t="inlineStr">
         <is>
-          <t>E-02 — A second player joins someone else's fight</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="19" customHeight="1">
+          <t>N-19 — Onslaught: random waves, surprise bosses, and no running away</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="49" customHeight="1">
       <c r="A102" s="15" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>N-19</t>
         </is>
       </c>
       <c r="B102" s="15" t="n">
@@ -5264,21 +5436,21 @@
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>Player one triggers N-08 or N-13</t>
+          <t>Type .nyar template use undead-onslaught, .nyar event enable undead-onslaught, then .nyar event start undead-onslaught in open ground</t>
         </is>
       </c>
       <c r="D102" s="15" t="inlineStr">
         <is>
-          <t>monsters hunt player one.</t>
+          <t>about 12 undead appear around you.</t>
         </is>
       </c>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="7" t="n"/>
     </row>
-    <row r="103" ht="19" customHeight="1">
+    <row r="103" ht="34" customHeight="1">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>N-19</t>
         </is>
       </c>
       <c r="B103" s="15" t="n">
@@ -5286,68 +5458,271 @@
       </c>
       <c r="C103" s="15" t="inlineStr">
         <is>
-          <t>Player two joins the fight and attacks the monsters</t>
+          <t>Clear wave 1 or wait 75 seconds</t>
         </is>
       </c>
       <c r="D103" s="15" t="inlineStr">
         <is>
-          <t>note who they turn on, and who gets kill credit.</t>
+          <t>wave 2 brings different undead and one V Blood boss.</t>
         </is>
       </c>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="7" t="n"/>
     </row>
-    <row r="104" ht="21" customHeight="1">
-      <c r="A104" s="18" t="inlineStr">
-        <is>
-          <t>C-01 — Measurement: how the server feels during the busiest event</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="49" customHeight="1">
+    <row r="104" ht="49" customHeight="1">
+      <c r="A104" s="15" t="inlineStr">
+        <is>
+          <t>N-19</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>Both players run more than 60 m away and wait</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>about a minute later the undead come after the nearest of you, arriving near you rather than on top of you.</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="n"/>
+      <c r="F104" s="7" t="n"/>
+    </row>
+    <row r="105" ht="19" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>C-01</t>
+          <t>N-19</t>
         </is>
       </c>
       <c r="B105" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C105" s="15" t="inlineStr">
         <is>
-          <t>At the start, at each horde rise and at the end, note how responsive the game feels (fine, slight lag, bad lag) and the time.</t>
-        </is>
-      </c>
-      <c r="D105" s="15" t="inlineStr"/>
+          <t>Go into your castle's territory</t>
+        </is>
+      </c>
+      <c r="D105" s="15" t="inlineStr">
+        <is>
+          <t>they do not follow you in.</t>
+        </is>
+      </c>
       <c r="E105" s="7" t="n"/>
       <c r="F105" s="7" t="n"/>
     </row>
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="15" t="inlineStr">
         <is>
-          <t>C-01</t>
+          <t>N-19</t>
         </is>
       </c>
       <c r="B106" s="15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C106" s="15" t="inlineStr">
         <is>
-          <t>If something felt bad, write what you were doing and how many monsters were around.</t>
-        </is>
-      </c>
-      <c r="D106" s="15" t="inlineStr"/>
+          <t>Stop it (.nyar event stop undead-onslaught) and start it again</t>
+        </is>
+      </c>
+      <c r="D106" s="15" t="inlineStr">
+        <is>
+          <t>the waves and bosses are different.</t>
+        </is>
+      </c>
       <c r="E106" s="7" t="n"/>
       <c r="F106" s="7" t="n"/>
     </row>
+    <row r="107" ht="21" customHeight="1">
+      <c r="A107" s="18" t="inlineStr">
+        <is>
+          <t>E-01 — Build your own event from chat, the way a new admin would</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="19" customHeight="1">
+      <c r="A108" s="15" t="inlineStr">
+        <is>
+          <t>E-01</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" s="15" t="inlineStr">
+        <is>
+          <t>Type .nyar event new my-event spawns</t>
+        </is>
+      </c>
+      <c r="D108" s="15" t="inlineStr">
+        <is>
+          <t>a switched-off event is created.</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n"/>
+      <c r="F108" s="7" t="n"/>
+    </row>
+    <row r="109" ht="49" customHeight="1">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>E-01</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C109" s="15" t="inlineStr">
+        <is>
+          <t>Use .nyar event set my-event ... to choose units (action.units, e.g. CHAR_Forest_Wolf:4), waves, the location (location here) and a level (action.modifiers.level 30).</t>
+        </is>
+      </c>
+      <c r="D109" s="15" t="inlineStr"/>
+      <c r="E109" s="7" t="n"/>
+      <c r="F109" s="7" t="n"/>
+    </row>
+    <row r="110" ht="19" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>E-01</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C110" s="15" t="inlineStr">
+        <is>
+          <t>Type .nyar event info my-event, then enable and start it</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="inlineStr">
+        <is>
+          <t>it runs as you set it.</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n"/>
+      <c r="F110" s="7" t="n"/>
+    </row>
+    <row r="111" ht="19" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>E-01</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C111" s="15" t="inlineStr">
+        <is>
+          <t>Note every reply that confused you, word for word.</t>
+        </is>
+      </c>
+      <c r="D111" s="15" t="inlineStr"/>
+      <c r="E111" s="7" t="n"/>
+      <c r="F111" s="7" t="n"/>
+    </row>
+    <row r="112" ht="21" customHeight="1">
+      <c r="A112" s="18" t="inlineStr">
+        <is>
+          <t>E-02 — A second player joins someone else's fight</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="19" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>E-02</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C113" s="15" t="inlineStr">
+        <is>
+          <t>Player one triggers N-08 or N-13</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr">
+        <is>
+          <t>monsters hunt player one.</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="n"/>
+      <c r="F113" s="7" t="n"/>
+    </row>
+    <row r="114" ht="19" customHeight="1">
+      <c r="A114" s="15" t="inlineStr">
+        <is>
+          <t>E-02</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C114" s="15" t="inlineStr">
+        <is>
+          <t>Player two joins the fight and attacks the monsters</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>note who they turn on, and who gets kill credit.</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="n"/>
+      <c r="F114" s="7" t="n"/>
+    </row>
+    <row r="115" ht="21" customHeight="1">
+      <c r="A115" s="18" t="inlineStr">
+        <is>
+          <t>C-01 — Measurement: how the server feels during the busiest event</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="49" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>C-01</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C116" s="15" t="inlineStr">
+        <is>
+          <t>At the start, at each horde rise and at the end, note how responsive the game feels (fine, slight lag, bad lag) and the time.</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr"/>
+      <c r="E116" s="7" t="n"/>
+      <c r="F116" s="7" t="n"/>
+    </row>
+    <row r="117" ht="34" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>C-01</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C117" s="15" t="inlineStr">
+        <is>
+          <t>If something felt bad, write what you were doing and how many monsters were around.</t>
+        </is>
+      </c>
+      <c r="D117" s="15" t="inlineStr"/>
+      <c r="E117" s="7" t="n"/>
+      <c r="F117" s="7" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F106"/>
-  <mergeCells count="20">
+  <autoFilter ref="A1:F117"/>
+  <mergeCells count="22">
     <mergeCell ref="A74:F74"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A56:F56"/>
     <mergeCell ref="A101:F101"/>
-    <mergeCell ref="A104:F104"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A62:F62"/>
@@ -5355,16 +5730,19 @@
     <mergeCell ref="A91:F91"/>
     <mergeCell ref="A29:F29"/>
     <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A115:F115"/>
+    <mergeCell ref="A112:F112"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A67:F67"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A107:F107"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A87:F87"/>
     <mergeCell ref="A7:F7"/>
   </mergeCells>
-  <conditionalFormatting sqref="E2:E106">
+  <conditionalFormatting sqref="E2:E117">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>E2="OK"</formula>
     </cfRule>
@@ -5376,7 +5754,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Problem,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5714,7 +6092,7 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF('Test plan'!$I$2:$I$21,"Pass")</f>
+        <f>COUNTIF('Test plan'!$I$2:$I$23,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5725,7 +6103,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test plan'!$I$2:$I$21,"Partial pass")</f>
+        <f>COUNTIF('Test plan'!$I$2:$I$23,"Partial pass")</f>
         <v/>
       </c>
     </row>
@@ -5736,7 +6114,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test plan'!$I$2:$I$21,"Fail")</f>
+        <f>COUNTIF('Test plan'!$I$2:$I$23,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5747,7 +6125,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test plan'!$I$2:$I$21,"Blocked")</f>
+        <f>COUNTIF('Test plan'!$I$2:$I$23,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5758,7 +6136,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test plan'!$I$2:$I$21,"Not tested yet")</f>
+        <f>COUNTIF('Test plan'!$I$2:$I$23,"Not tested yet")</f>
         <v/>
       </c>
     </row>
@@ -5769,7 +6147,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTA('Test plan'!$A$2:$A$21)</f>
+        <f>COUNTA('Test plan'!$A$2:$A$23)</f>
         <v/>
       </c>
     </row>
@@ -5787,7 +6165,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIF('Test plan'!$H$2:$H$21,"Tester A")</f>
+        <f>COUNTIF('Test plan'!$H$2:$H$23,"Tester A")</f>
         <v/>
       </c>
     </row>
@@ -5798,7 +6176,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF('Test plan'!$H$2:$H$21,"Tester B")</f>
+        <f>COUNTIF('Test plan'!$H$2:$H$23,"Tester B")</f>
         <v/>
       </c>
     </row>
@@ -5809,7 +6187,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF('Test plan'!$H$2:$H$21,"Both — coordinated")</f>
+        <f>COUNTIF('Test plan'!$H$2:$H$23,"Both — coordinated")</f>
         <v/>
       </c>
     </row>
@@ -5820,7 +6198,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF('Test plan'!$H$2:$H$21,"Not assigned yet")</f>
+        <f>COUNTIF('Test plan'!$H$2:$H$23,"Not assigned yet")</f>
         <v/>
       </c>
     </row>
@@ -5831,7 +6209,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTBLANK('Test plan'!$H$2:$H$21)</f>
+        <f>COUNTBLANK('Test plan'!$H$2:$H$23)</f>
         <v/>
       </c>
     </row>
@@ -5849,7 +6227,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIF('Test plan'!$B$2:$B$21,"New")</f>
+        <f>COUNTIF('Test plan'!$B$2:$B$23,"New")</f>
         <v/>
       </c>
     </row>
@@ -5860,7 +6238,7 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF('Test plan'!$B$2:$B$21,"Established feature — a fresh pair of eyes")</f>
+        <f>COUNTIF('Test plan'!$B$2:$B$23,"Established feature — a fresh pair of eyes")</f>
         <v/>
       </c>
     </row>
@@ -5871,7 +6249,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF('Test plan'!$B$2:$B$21,"Not an ordinary test row")</f>
+        <f>COUNTIF('Test plan'!$B$2:$B$23,"Not an ordinary test row")</f>
         <v/>
       </c>
     </row>
@@ -5889,7 +6267,7 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIF('Test steps'!$E$2:$E$106,"OK")</f>
+        <f>COUNTIF('Test steps'!$E$2:$E$117,"OK")</f>
         <v/>
       </c>
     </row>
@@ -5900,7 +6278,7 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIF('Test steps'!$E$2:$E$106,"Problem")</f>
+        <f>COUNTIF('Test steps'!$E$2:$E$117,"Problem")</f>
         <v/>
       </c>
     </row>
@@ -5911,7 +6289,7 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Test steps'!$E$2:$E$106,"Skipped")</f>
+        <f>COUNTIF('Test steps'!$E$2:$E$117,"Skipped")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(testing): rows set events up as a live server would (rc.3 round 1)
Saved spots (location here) for the ambush, timed and onslaught rows, a
scheduled and announced arena night, a named place to defend for the
apocalypse, event banners on in the install steps. tester-setups.vrs
covers every new setup command (79/80 on rc.3; the refused arena step
was dropped).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMjJ2LeCjs6pJ2deXkbdAT
</commit_message>
<xml_diff>
--- a/testing/nyarlathotep-dev-round-01-production-setups.xlsx
+++ b/testing/nyarlathotep-dev-round-01-production-setups.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test plan'!$A$1:$P$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test steps'!$A$1:$F$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test steps'!$A$1:$F$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -673,511 +673,518 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>7. Make each tester an admin: add their Steam ID (the 17-digit number) on its own line to adminlist.txt in the server's save data Settings folder, then restart the server -&gt; in game, with the console switched on in Options, press the ~ key and type adminauth.</t>
+          <t>7. So players see events as they would on a live server: stop the server, open BepInEx/config/kdpen.Nyarlathotep.cfg, set EventBanners = true under [Announcements], save, start the server -&gt; from now on everyone gets a server-wide line when an event starts and when it ends.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>8. In game, type .nyar in chat -&gt; the first line reads 'Nyarlathotep, Lord of Chaos (v0.13.0-rc.3)' and the admin commands are listed. Everything ships switched off; each row turns on what it needs.</t>
+          <t>8. Make each tester an admin: add their Steam ID (the 17-digit number) on its own line to adminlist.txt in the server's save data Settings folder, then restart the server -&gt; in game, with the console switched on in Options, press the ~ key and type adminauth.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>9. For a newer test build later: stop the server, replace Nyarlathotep.dll, start it -&gt; the version line shows the new build. To remove the mod: type .nyar purge then .nyar purge confirm, stop the server, delete the file -&gt; no monster of ours is left behind.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="19" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+          <t>9. In game, type .nyar in chat -&gt; the first line reads 'Nyarlathotep, Lord of Chaos (v0.13.0-rc.3)' and the admin commands are listed. Everything ships switched off; each row turns on what it needs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>10. For a newer test build later: stop the server, replace Nyarlathotep.dll, start it -&gt; the version line shows the new build. To remove the mod: type .nyar purge then .nyar purge confirm, stop the server, delete the file -&gt; no monster of ours is left behind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Tester details — one column each. The line under each field says why we ask.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Tester A</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Tester B</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Why we ask</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="49" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="19" ht="49" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Name</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>So we know whose notes these are when two of you return one file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="64" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Timezone</t>
         </is>
       </c>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Schedules run on the server's clock; your own time zone explains a 'wrong hour' report.</t>
+          <t>So we know whose notes these are when two of you return one file.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="64" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>PC (make, model, rough age)</t>
+          <t>Timezone</t>
         </is>
       </c>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Frame drops during large fights depend on the machine as much as the server.</t>
+          <t>Schedules run on the server's clock; your own time zone explains a 'wrong hour' report.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="64" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Windows version</t>
+          <t>PC (make, model, rough age)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Rarely matters for a server mod, but costs nothing and closes a question.</t>
+          <t>Frame drops during large fights depend on the machine as much as the server.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="64" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>V Rising version (title screen)</t>
+          <t>Windows version</t>
         </is>
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>A client older than the server cannot join; it also ties a report to a game patch.</t>
+          <t>Rarely matters for a server mod, but costs nothing and closes a question.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="64" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Display size and scaling</t>
+          <t>V Rising version (title screen)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Chat lines can wrap or clip at high scaling; a cut-off line is otherwise unattributable.</t>
+          <t>A client older than the server cannot join; it also ties a report to a game patch.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="64" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Input (mouse and keyboard, controller)</t>
+          <t>Display size and scaling</t>
         </is>
       </c>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Some rows ask you to climb, kite or stand still; input changes how that goes.</t>
+          <t>Chat lines can wrap or clip at high scaling; a cut-off line is otherwise unattributable.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="64" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Connection (wired, wifi, rough ping)</t>
+          <t>Input (mouse and keyboard, controller)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n"/>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Units that jump or rubber-band can be lag on your side rather than the mod.</t>
+          <t>Some rows ask you to climb, kite or stand still; input changes how that goes.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="64" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Character gear level at start</t>
+          <t>Connection (wired, wifi, rough ping)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Event difficulty is set by level; your level explains 'too easy' or 'too hard'.</t>
+          <t>Units that jump or rubber-band can be lag on your side rather than the mod.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="64" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Admin on the dev server? (yes or no)</t>
+          <t>Character gear level at start</t>
         </is>
       </c>
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Setting up events needs admin rights; rows marked admin come back Blocked without them.</t>
+          <t>Event difficulty is set by level; your level explains 'too easy' or 'too hard'.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="64" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Date started</t>
+          <t>Admin on the dev server? (yes or no)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Ties the round to a build; the dev server may be updated during the round.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="19" customHeight="1">
+          <t>Setting up events needs admin rights; rows marked admin come back Blocked without them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="64" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Date finished</t>
+          <t>Date started</t>
         </is>
       </c>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>As above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="49" customHeight="1">
+          <t>Ties the round to a build; the dev server may be updated during the round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Rough hours spent</t>
+          <t>Date finished</t>
         </is>
       </c>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="6" t="inlineStr">
         <is>
+          <t>As above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="49" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Rough hours spent</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
           <t>Tells us whether the round is the right size for next time.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="33" ht="19" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Where your last round's findings went</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="34" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>This is the first round, so there are no earlier findings to account for. From round two, this block lists every finding you sent, by your reference, and what happened to it.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="35" ht="19" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>What we could not check ourselves, and why</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="34" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>• Anything that needs a second player. Our own test tool plays one character alone, and it is invulnerable, so monsters never truly chase it. Every row that needs two of you says so.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="34" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>• A real player in danger. Because our character cannot be hurt, we could never see a monster that wants to reach a player but cannot (the stuck-unit rows), or how an ambush feels when it can actually kill you.</t>
+          <t>• Anything that needs a second player. Our own test tool plays one character alone, and it is invulnerable, so monsters never truly chase it. Every row that needs two of you says so.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="34" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>• How it feels. Whether a fight is fun, an announcement reads well, a jump looks natural, or the server stays smooth while a hundred monsters roam: only people playing can judge that.</t>
+          <t>• A real player in danger. Because our character cannot be hurt, we could never see a monster that wants to reach a player but cannot (the stuck-unit rows), or how an ambush feels when it can actually kill you.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="34" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>• How it feels. Whether a fight is fun, an announcement reads well, a jump looks natural, or the server stays smooth while a hundred monsters roam: only people playing can judge that.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>• Real triggers. We start events by command. A schedule, nightfall, a V Blood kill, walking into a region and killing a faction's people are the ways events start on a real server, and they need real play.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="19" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="40" ht="19" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Your access</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="49" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="41" ht="49" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Connect to the dev server, the test server set up with the steps under 'Installing the build', at the address its admin gives you (Direct Connect, not the server list). 20 of the 22 rows need admin rights: the owner adds you as an admin before the round, and you type '.nyar' in chat to confirm you see the admin commands. Rows that need admin say so under 'You will need'.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="19" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
+    <row r="43" ht="19" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>How this workbook works</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="19" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>• What changed: read first: every row, what it is and how to check it. Nothing to type.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="19" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>• Known limits: what will look like a fault and is not. Read before starting.</t>
+          <t>• What changed: read first: every row, what it is and how to check it. Nothing to type.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="19" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>• Test plan: one line per test: your result goes here.</t>
+          <t>• Known limits: what will look like a fault and is not. Read before starting.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="19" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>• Test steps: every step of every test, each with OK, Problem or Skipped.</t>
+          <t>• Test plan: one line per test: your result goes here.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="19" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>• Anything new: anything you notice that is not on a row.</t>
+          <t>• Test steps: every step of every test, each with OK, Problem or Skipped.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="19" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>• Anything new: anything you notice that is not on a row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="19" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>• Progress: counts itself. Nothing to fill in.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="19" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+    <row r="50" ht="19" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>Results (Test plan)</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="19" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="51" ht="19" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>• Pass: Does what the row says, and nothing bothered you.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="19" customHeight="1">
-      <c r="A51" s="9" t="inlineStr">
+    <row r="52" ht="19" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>• Partial pass: Anything in between: most steps work and one does not, or it works but something else went wrong.</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="19" customHeight="1">
-      <c r="A52" s="10" t="inlineStr">
+    <row r="53" ht="19" customHeight="1">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>• Fail: Does not do what the row says.</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="19" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+    <row r="54" ht="19" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>• Blocked: Could not reach it: no second player, no admin rights, the server was down.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="19" customHeight="1">
-      <c r="A54" s="12" t="inlineStr">
+    <row r="55" ht="19" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>• Not tested yet: Nobody has started it.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="19" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+    <row r="56" ht="19" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Step results (Test steps)</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="19" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="57" ht="19" customHeight="1">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>• OK: The step did what it says.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="19" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
+    <row r="58" ht="19" customHeight="1">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>• Problem: It did not, or something odd happened.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="19" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="59" ht="19" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>• Skipped: You could not do this step.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="19" customHeight="1">
-      <c r="A59" s="3" t="inlineStr">
+    <row r="60" ht="19" customHeight="1">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Row categories, in the order you meet them</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="19" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>• New</t>
         </is>
       </c>
     </row>
     <row r="61" ht="19" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>• Established feature — a fresh pair of eyes</t>
+          <t>• New</t>
         </is>
       </c>
     </row>
     <row r="62" ht="19" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>• Established feature — a fresh pair of eyes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="19" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
           <t>• Not an ordinary test row</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="19" customHeight="1">
-      <c r="A63" s="3" t="inlineStr">
+    <row r="64" ht="19" customHeight="1">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>Reporting rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="19" customHeight="1">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>• Put a name against every row in 'Assigned to' before either of you begins.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="19" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>• Fill in 'Tested at' (date and time) on every row you test.</t>
+          <t>• Put a name against every row in 'Assigned to' before either of you begins.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="19" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>• If a row is not a clean Pass, fill in 'If not a clean pass — what is still wrong'. It is not optional.</t>
+          <t>• Fill in 'Tested at' (date and time) on every row you test.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="19" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>• Say so plainly if something is wrong. A finding we disagree with is still worth having; give the evidence (a screenshot, the exact chat line) if you have it.</t>
+          <t>• If a row is not a clean Pass, fill in 'If not a clean pass — what is still wrong'. It is not optional.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="19" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>• If the two of you disagree about whether something is a fault, put both views in. A disagreement is a finding.</t>
+          <t>• Say so plainly if something is wrong. A finding we disagree with is still worth having; give the evidence (a screenshot, the exact chat line) if you have it.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="19" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>• Anything not on a row goes on 'Anything new'. Small things are welcome.</t>
+          <t>• If the two of you disagree about whether something is a fault, put both views in. A disagreement is a finding.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="19" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>• Blocked is a real answer. If a row needs a second player or admin rights you do not have, mark it Blocked and move on rather than improvising.</t>
+          <t>• Anything not on a row goes on 'Anything new'. Small things are welcome.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="19" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
+          <t>• Blocked is a real answer. If a row needs a second player or admin rights you do not have, mark it Blocked and move on rather than improvising.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="19" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
           <t>• Chat commands are typed exactly as written, including the dot at the start. Text in angle brackets, such as &lt;id&gt;, is replaced by the value named.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="53">
-    <mergeCell ref="A16:F16"/>
+  <mergeCells count="54">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="A66:F66"/>
@@ -1192,14 +1199,14 @@
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A71:F71"/>
     <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A72:F72"/>
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A63:F63"/>
@@ -1215,8 +1222,9 @@
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A64:F64"/>
-    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="A51:F51"/>
@@ -1356,7 +1364,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="79" customHeight="1">
+    <row r="5" ht="64" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
           <t>N-03</t>
@@ -1379,12 +1387,12 @@
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>The 'Legion weekend surge' template empowers the Legion on Saturdays at 20:00. Here you move its time to a few minutes from now, as an admin planning a real evening would.</t>
+          <t>'Legion weekend surge' empowers the Legion on Saturdays at 20:00. Here you move its time to a few minutes from now, as an admin planning a real evening would.</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use legion-weekend-surge, then .nyar event enable legion-weekend-surge.</t>
+          <t>Type .nyar template use legion-weekend-surge and .nyar pillar empowerment on.</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1441,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>An admin-run ambush at a bandit camp</t>
+          <t>An ambush waiting at a spot you choose</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -1443,12 +1451,12 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>'Bandit ambush' brings 3 waves of bandit thugs and hunters around the admin, a minute apart: the kind of event an admin starts by hand for a group evening.</t>
+          <t>The admin picks the place first and can then start the event from anywhere. 'Bandit ambush' brings 3 waves of bandits to the saved spot, a minute apart.</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use bandit-ambush, .nyar pillar spawns on, .nyar event enable bandit-ambush.</t>
+          <t>Type .nyar template use bandit-ambush and .nyar pillar spawns on</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1588,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="79" customHeight="1">
+    <row r="12" ht="94" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
         <is>
           <t>N-10</t>
@@ -1593,7 +1601,7 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Spider swarm: an arena, growing waves and the Spider Queen</t>
+          <t>A scheduled arena night: the spider swarm at a set place and time</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -1603,12 +1611,12 @@
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>'Spider swarm' holds 5 waves of spiders in a 40 m arena around where the admin starts it; each wave adds a spider and 3 levels, the last brings the Spider Queen. The best kills-to-deaths ratio wins.</t>
+          <t>How a server runs a weekly event: the admin picks the arena, sets the day and time and tells the players. The swarm then starts by itself: 5 growing waves in the arena, the Spider Queen last, and the best kills-to-deaths ratio wins.</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use spider-swarm, .nyar event enable spider-swarm, then .nyar event info spider-swarm</t>
+          <t>Type .nyar template use spider-swarm. Stand in the middle of your arena and type .nyar event set spider-swarm location here</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1716,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="79" customHeight="1">
+    <row r="16" ht="94" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
           <t>N-14</t>
@@ -1731,12 +1739,12 @@
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>The undead rise at three hotspots, roamers hunt players across the map and spread with every kill, and four hordes march on the spot the admin defends. The last horde brings the Bishop of Death.</t>
+          <t>The undead rise at three hotspots, roamers hunt players across the map and spread with every kill, and four hordes march on a place the admin names for the server to defend. The last horde brings the Bishop of Death.</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use zombie-apocalypse, .nyar event enable zombie-apocalypse, and .nyar event set zombie-apocalypse durationSeconds 7200.</t>
+          <t>Type .nyar template use zombie-apocalypse and .nyar event set zombie-apocalypse durationSeconds 7200.</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1780,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="49" customHeight="1">
+    <row r="18" ht="64" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
           <t>N-16</t>
@@ -1800,7 +1808,7 @@
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>Stand inside your castle territory. Type .nyar event start bandit-ambush (set up in N-05)</t>
+          <t>Stand inside your castle territory with nobody else online outside one. Type .nyar event start graveyard-waves (set up in N-06)</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1844,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="109" customHeight="1">
+    <row r="20" ht="94" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
           <t>N-18</t>
@@ -1849,7 +1857,7 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>Timed waves: the next wave comes whether you are ready or not</t>
+          <t>Timed waves at a muster point: the next wave comes whether you are ready or not</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1859,12 +1867,12 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>'Militia muster (timed)' is militia-muster on a clock: 5 waves of militia in a 40 m arena, a new wave every 75 seconds even if the last one is still alive, ending on the militia leader. Six other factions have a timed version too (names ending in -timed).</t>
+          <t>'Militia muster (timed)' brings 5 waves of militia to a place the admin saves, a new wave every 75 seconds even if the last is still alive, ending on the militia leader. Six other factions have a timed version too (names ending in -timed).</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use militia-muster-timed, .nyar event enable militia-muster-timed.</t>
+          <t>Type .nyar template use militia-muster-timed. At an open spot in Dunley Farmlands type .nyar event set militia-muster-timed location here</t>
         </is>
       </c>
     </row>
@@ -1891,12 +1899,12 @@
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>'Undead onslaught' rolls each wave at random from groups of undead, adds a random undead V Blood in the middle wave and one or two at the end. If nobody stays in the 40 m arena for 60 seconds, the undead go after the nearest player anywhere on the map. Six other factions have one too (names ending in -onslaught).</t>
+          <t>'Undead onslaught' rolls each wave at random from groups of undead, adds a random undead V Blood in the middle wave and one or two at the end. If nobody stays in its 40 m arena, after a set time the undead go after the nearest player anywhere on the map. Six other factions have one too (names ending in -onslaught).</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use undead-onslaught, .nyar event enable undead-onslaught, then .nyar event start undead-onslaught in open ground</t>
+          <t>Type .nyar template use undead-onslaught. At an open spot near a graveyard type .nyar event set undead-onslaught location here.</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2569,7 @@
       <c r="O5" s="17" t="n"/>
       <c r="P5" s="17" t="n"/>
     </row>
-    <row r="6" ht="49" customHeight="1">
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
           <t>N-05</t>
@@ -2579,20 +2587,20 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>An admin-run ambush at a bandit camp</t>
+          <t>An ambush waiting at a spot you choose</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>Admin rights; one or two players with gear level 20 or more; open ground away from any castle.</t>
+          <t>Admin rights; one or two players with gear level 25 or more; a road or clearing away from any castle.</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>Did the waves arrive on walkable ground near you, never inside rocks or water?</t>
+          <t>Were the bandits at the saved spot, on walkable ground, and at the level you set?</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -2821,7 +2829,7 @@
       <c r="O10" s="17" t="n"/>
       <c r="P10" s="17" t="n"/>
     </row>
-    <row r="11" ht="49" customHeight="1">
+    <row r="11" ht="79" customHeight="1">
       <c r="A11" s="15" t="inlineStr">
         <is>
           <t>N-10</t>
@@ -2839,12 +2847,12 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>Spider swarm: an arena, growing waves and the Spider Queen</t>
+          <t>A scheduled arena night: the spider swarm at a set place and time</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>Admin rights; two players with gear level 35 or more (the Queen is level 45); open ground.</t>
+          <t>Admin rights; the server's local time; two players with gear level 35 or more (the Queen is level 45); open ground away from castles.</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
@@ -2852,7 +2860,7 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>Did the arena edge feel fair, or did spiders snap back in a way that looked wrong?</t>
+          <t>Could you run a real arena night this way, and did the arena edge feel fair?</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
@@ -3029,7 +3037,7 @@
       <c r="O14" s="17" t="n"/>
       <c r="P14" s="17" t="n"/>
     </row>
-    <row r="15" ht="64" customHeight="1">
+    <row r="15" ht="79" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
           <t>N-14</t>
@@ -3052,7 +3060,7 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>Admin rights; two hours; as many players as you can gather, gear level 30 or more; a spot to defend outside any castle.</t>
+          <t>Admin rights; two hours; as many players as you can gather, gear level 30 or more; a place to defend outside any castle (a crossroads, a ruin).</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
@@ -3237,7 +3245,7 @@
       <c r="O18" s="17" t="n"/>
       <c r="P18" s="17" t="n"/>
     </row>
-    <row r="19" ht="79" customHeight="1">
+    <row r="19" ht="94" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
           <t>N-18</t>
@@ -3255,16 +3263,16 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Timed waves: the next wave comes whether you are ready or not</t>
+          <t>Timed waves at a muster point: the next wave comes whether you are ready or not</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>Admin rights; the Spawns kind on (.nyar pillar spawns on); two players with gear level 50 or more (the militia leader is level 58); open ground.</t>
+          <t>Admin rights; the Spawns kind on (.nyar pillar spawns on); two players with gear level 50 or more (the militia leader is level 58); open ground in Dunley Farmlands.</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
@@ -3289,7 +3297,7 @@
       <c r="O19" s="17" t="n"/>
       <c r="P19" s="17" t="n"/>
     </row>
-    <row r="20" ht="79" customHeight="1">
+    <row r="20" ht="94" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
           <t>N-19</t>
@@ -3312,7 +3320,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Admin rights; the Spawns kind on; two players with gear level 60 or more (the undead V Bloods run from level 27 to 63, up to two at once); a castle nearby.</t>
+          <t>Admin rights; the Spawns kind on; two players with gear level 60 or more (the undead V Bloods run from level 27 to 63, up to two at once); a castle within reach.</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
@@ -3535,7 +3543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F117"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3808,14 +3816,14 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use legion-weekend-surge, then .nyar event enable legion-weekend-surge.</t>
+          <t>Type .nyar template use legion-weekend-surge and .nyar pillar empowerment on.</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
     </row>
-    <row r="15" ht="34" customHeight="1">
+    <row r="15" ht="49" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
           <t>N-03</t>
@@ -3826,12 +3834,12 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event set legion-weekend-surge trigger.days &lt;today, e.g. Wed&gt;</t>
+          <t>Type .nyar event set legion-weekend-surge trigger.days &lt;today, e.g. Wed&gt; and .nyar event set legion-weekend-surge trigger.times &lt;server time plus 5 minutes, e.g. 21:35&gt;</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>it confirms.</t>
+          <t>each confirms.</t>
         </is>
       </c>
       <c r="E15" s="7" t="n"/>
@@ -3848,12 +3856,12 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event set legion-weekend-surge trigger.times &lt;server time plus 5 minutes, e.g. 21:35&gt;</t>
+          <t>Type .nyar event enable legion-weekend-surge, then .nyar event info legion-weekend-surge</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>it confirms; .nyar event info legion-weekend-surge shows the next start.</t>
+          <t>it shows the next start.</t>
         </is>
       </c>
       <c r="E16" s="7" t="n"/>
@@ -3997,7 +4005,7 @@
     <row r="24" ht="21" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>N-05 — An admin-run ambush at a bandit camp</t>
+          <t>N-05 — An ambush waiting at a spot you choose</t>
         </is>
       </c>
     </row>
@@ -4012,10 +4020,14 @@
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use bandit-ambush, .nyar pillar spawns on, .nyar event enable bandit-ambush.</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="inlineStr"/>
+          <t>Type .nyar template use bandit-ambush and .nyar pillar spawns on</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>both confirm.</t>
+        </is>
+      </c>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="7" t="n"/>
     </row>
@@ -4030,18 +4042,18 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Stand where the ambush should happen and type .nyar event start bandit-ambush</t>
+          <t>Walk to where the ambush should happen and type .nyar event set bandit-ambush location here</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>a start line shows; about 6 bandits appear within 10 m.</t>
+          <t>it confirms with your position.</t>
         </is>
       </c>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="7" t="n"/>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="49" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
           <t>N-05</t>
@@ -4052,18 +4064,18 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Fight them</t>
+          <t>Set the difficulty with .nyar event set bandit-ambush action.modifiers.level 30, then type .nyar event enable bandit-ambush</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>a second and third wave arrive a minute apart.</t>
+          <t>each confirms.</t>
         </is>
       </c>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="7" t="n"/>
     </row>
-    <row r="28" ht="49" customHeight="1">
+    <row r="28" ht="34" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
           <t>N-05</t>
@@ -4074,41 +4086,45 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>After 10 minutes, or when you type .nyar event stop bandit-ambush</t>
+          <t>Walk at least 100 m away and type .nyar event start bandit-ambush</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>an end line shows; any bandits left disappear about 30 s later; .nyar status reads 'tracked units: 0'.</t>
+          <t>nothing appears around you; the bandits are waiting at the saved spot.</t>
         </is>
       </c>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="7" t="n"/>
     </row>
-    <row r="29" ht="21" customHeight="1">
-      <c r="A29" s="18" t="inlineStr">
+    <row r="29" ht="79" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>N-05</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>Go back and fight</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>waves 2 and 3 arrive a minute apart, all at level 30. When it ends (10 minutes, or .nyar event stop bandit-ambush) the leftovers disappear about 30 s later; .nyar status reads 'tracked units: 0'.</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+    </row>
+    <row r="30" ht="21" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>N-06 — Graveyard waves: three waves, a guardian and a scoreboard</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="34" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>N-06</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar template use graveyard-waves, .nyar event enable graveyard-waves.</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
     </row>
     <row r="31" ht="34" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
@@ -4117,18 +4133,14 @@
         </is>
       </c>
       <c r="B31" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Everyone goes to a graveyard (outside castles); the admin types .nyar event start graveyard-waves</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="inlineStr">
-        <is>
-          <t>skeletons appear 20-40 m from one player and come for you.</t>
-        </is>
-      </c>
+          <t>Type .nyar template use graveyard-waves, .nyar event enable graveyard-waves.</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
     </row>
@@ -4139,16 +4151,16 @@
         </is>
       </c>
       <c r="B32" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Clear wave 1</t>
+          <t>Everyone goes to a graveyard (outside castles); the admin types .nyar event start graveyard-waves</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>wave 2 comes (stronger), then wave 3 with the Undead Guardian.</t>
+          <t>skeletons appear 20-40 m from one player and come for you.</t>
         </is>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -4161,101 +4173,101 @@
         </is>
       </c>
       <c r="B33" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Clear wave 3</t>
+          <t>Clear wave 1</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>chat says all waves are defeated and shows the top 3 by kills with deaths.</t>
+          <t>wave 2 comes (stronger), then wave 3 with the Undead Guardian.</t>
         </is>
       </c>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
     </row>
-    <row r="34" ht="19" customHeight="1">
+    <row r="34" ht="34" customHeight="1">
       <c r="A34" s="15" t="inlineStr">
         <is>
           <t>N-06</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Compare the scoreboard with who actually got the kills.</t>
-        </is>
-      </c>
-      <c r="D34" s="15" t="inlineStr"/>
+          <t>Clear wave 3</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>chat says all waves are defeated and shows the top 3 by kills with deaths.</t>
+        </is>
+      </c>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="n"/>
     </row>
-    <row r="35" ht="21" customHeight="1">
-      <c r="A35" s="18" t="inlineStr">
+    <row r="35" ht="19" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>N-06</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>Compare the scoreboard with who actually got the kills.</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+    </row>
+    <row r="36" ht="21" customHeight="1">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>N-07 — Hunters that roam on their own (a random interval) and split up between players</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="15" t="inlineStr">
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>N-07</t>
         </is>
       </c>
-      <c r="B36" s="15" t="n">
+      <c r="B37" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
         <is>
           <t>Type .nyar template use roaming-hunters, .nyar event enable roaming-hunters.</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-    </row>
-    <row r="37" ht="49" customHeight="1">
-      <c r="A37" s="15" t="inlineStr">
-        <is>
-          <t>N-07</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar event set roaming-hunters trigger.minMinutes 5 and .nyar event set roaming-hunters trigger.maxMinutes 5; .nyar event info roaming-hunters shows the next start.</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr"/>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
     </row>
-    <row r="38" ht="34" customHeight="1">
+    <row r="38" ht="49" customHeight="1">
       <c r="A38" s="15" t="inlineStr">
         <is>
           <t>N-07</t>
         </is>
       </c>
       <c r="B38" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Both players stand 150 m or more apart, outside castles</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>within about 5 minutes each of you gets a separate bandit squad 20-40 m away that hunts you.</t>
-        </is>
-      </c>
+          <t>Type .nyar event set roaming-hunters trigger.minMinutes 5 and .nyar event set roaming-hunters trigger.maxMinutes 5; .nyar event info roaming-hunters shows the next start.</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
     </row>
@@ -4266,45 +4278,49 @@
         </is>
       </c>
       <c r="B39" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>One player stands inside their castle territory at the next start</t>
+          <t>Both players stand 150 m or more apart, outside castles</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>that player gets no squad.</t>
+          <t>within about 5 minutes each of you gets a separate bandit squad 20-40 m away that hunts you.</t>
         </is>
       </c>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
     </row>
-    <row r="40" ht="21" customHeight="1">
-      <c r="A40" s="18" t="inlineStr">
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>N-07</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>One player stands inside their castle territory at the next start</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>that player gets no squad.</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
+    </row>
+    <row r="41" ht="21" customHeight="1">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>N-08 — The border watch rides out when you enter Dunley Farmlands</t>
         </is>
       </c>
-    </row>
-    <row r="41" ht="34" customHeight="1">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>N-08</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar template use border-watch, .nyar event enable border-watch.</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr"/>
-      <c r="E41" s="7" t="n"/>
-      <c r="F41" s="7" t="n"/>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="15" t="inlineStr">
@@ -4313,38 +4329,34 @@
         </is>
       </c>
       <c r="B42" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Walk across the border into Dunley Farmlands</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>within seconds militia appear 20-40 m away and hunt you.</t>
-        </is>
-      </c>
+          <t>Type .nyar template use border-watch, .nyar event enable border-watch.</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr"/>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="7" t="n"/>
     </row>
-    <row r="43" ht="19" customHeight="1">
+    <row r="43" ht="34" customHeight="1">
       <c r="A43" s="15" t="inlineStr">
         <is>
           <t>N-08</t>
         </is>
       </c>
       <c r="B43" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar region here</t>
+          <t>Walk across the border into Dunley Farmlands</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>it names Dunley Farmlands.</t>
+          <t>within seconds militia appear 20-40 m away and hunt you.</t>
         </is>
       </c>
       <c r="E43" s="7" t="n"/>
@@ -4357,45 +4369,49 @@
         </is>
       </c>
       <c r="B44" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Leave and walk back in within 30 minutes</t>
+          <t>Type .nyar region here</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>nothing spawns the second time.</t>
+          <t>it names Dunley Farmlands.</t>
         </is>
       </c>
       <c r="E44" s="7" t="n"/>
       <c r="F44" s="7" t="n"/>
     </row>
-    <row r="45" ht="21" customHeight="1">
-      <c r="A45" s="18" t="inlineStr">
+    <row r="45" ht="19" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>N-08</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>Leave and walk back in within 30 minutes</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>nothing spawns the second time.</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n"/>
+      <c r="F45" s="7" t="n"/>
+    </row>
+    <row r="46" ht="21" customHeight="1">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>N-09 — Bandit reprisal after a killing spree</t>
         </is>
       </c>
-    </row>
-    <row r="46" ht="34" customHeight="1">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>N-09</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar template use bandit-reprisal, .nyar event enable bandit-reprisal.</t>
-        </is>
-      </c>
-      <c r="D46" s="15" t="inlineStr"/>
-      <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="n"/>
     </row>
     <row r="47" ht="34" customHeight="1">
       <c r="A47" s="15" t="inlineStr">
@@ -4404,11 +4420,11 @@
         </is>
       </c>
       <c r="B47" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event set bandit-reprisal trigger.kills 10 and .nyar event set bandit-reprisal trigger.windowSeconds 600.</t>
+          <t>Type .nyar template use bandit-reprisal, .nyar event enable bandit-reprisal.</t>
         </is>
       </c>
       <c r="D47" s="15" t="inlineStr"/>
@@ -4422,111 +4438,107 @@
         </is>
       </c>
       <c r="B48" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Kill 10 bandits within 10 minutes</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>right after the tenth, a squad appears 20-40 m away and hunts you.</t>
-        </is>
-      </c>
+          <t>Type .nyar event set bandit-reprisal trigger.kills 10 and .nyar event set bandit-reprisal trigger.windowSeconds 600.</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr"/>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="7" t="n"/>
     </row>
-    <row r="49" ht="19" customHeight="1">
+    <row r="49" ht="34" customHeight="1">
       <c r="A49" s="15" t="inlineStr">
         <is>
           <t>N-09</t>
         </is>
       </c>
       <c r="B49" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>A second player kills only 5 bandits</t>
+          <t>Kill 10 bandits within 10 minutes</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>no squad comes for them.</t>
+          <t>right after the tenth, a squad appears 20-40 m away and hunts you.</t>
         </is>
       </c>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="7" t="n"/>
     </row>
-    <row r="50" ht="21" customHeight="1">
-      <c r="A50" s="18" t="inlineStr">
-        <is>
-          <t>N-10 — Spider swarm: an arena, growing waves and the Spider Queen</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="34" customHeight="1">
-      <c r="A51" s="15" t="inlineStr">
+    <row r="50" ht="19" customHeight="1">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>N-09</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>A second player kills only 5 bandits</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>no squad comes for them.</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="21" customHeight="1">
+      <c r="A51" s="18" t="inlineStr">
+        <is>
+          <t>N-10 — A scheduled arena night: the spider swarm at a set place and time</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="49" customHeight="1">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>N-10</t>
         </is>
       </c>
-      <c r="B51" s="15" t="n">
+      <c r="B52" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C51" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar template use spider-swarm, .nyar event enable spider-swarm, then .nyar event info spider-swarm</t>
-        </is>
-      </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>all five waves are listed with their counts and levels.</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="n"/>
-      <c r="F51" s="7" t="n"/>
-    </row>
-    <row r="52" ht="34" customHeight="1">
-      <c r="A52" s="15" t="inlineStr">
-        <is>
-          <t>N-10</t>
-        </is>
-      </c>
-      <c r="B52" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Stand in the middle of open ground and type .nyar event start spider-swarm</t>
+          <t>Type .nyar template use spider-swarm. Stand in the middle of your arena and type .nyar event set spider-swarm location here</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>spiders appear around you.</t>
+          <t>it confirms; the arena is the 40 m around that spot.</t>
         </is>
       </c>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="7" t="n"/>
     </row>
-    <row r="53" ht="19" customHeight="1">
+    <row r="53" ht="79" customHeight="1">
       <c r="A53" s="15" t="inlineStr">
         <is>
           <t>N-10</t>
         </is>
       </c>
       <c r="B53" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>Run more than 40 m from the centre during a wave</t>
+          <t>Type .nyar event set spider-swarm trigger.type Schedule, .nyar event set spider-swarm trigger.days &lt;today, e.g. Sat&gt; and .nyar event set spider-swarm trigger.times &lt;server time plus 10 minutes, e.g. 21:40&gt;, then .nyar event enable spider-swarm</t>
         </is>
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>the spiders do not follow you out; they go back.</t>
+          <t>.nyar event info spider-swarm shows the next start and all five waves.</t>
         </is>
       </c>
       <c r="E53" s="7" t="n"/>
@@ -4539,16 +4551,16 @@
         </is>
       </c>
       <c r="B54" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Clear the waves</t>
+          <t>Tell everyone: .nyar announce Spider arena at &lt;place&gt; in 10 minutes</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>each one is bigger; wave 5 brings the Spider Queen.</t>
+          <t>every player sees the line.</t>
         </is>
       </c>
       <c r="E54" s="7" t="n"/>
@@ -4561,65 +4573,65 @@
         </is>
       </c>
       <c r="B55" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Kill the Queen</t>
+          <t>Gather in the arena; nobody types start</t>
         </is>
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>chat shows the scoreboard and names a winner; you can feed on the Queen's V Blood.</t>
+          <t>on the minute, a start line shows and spiders appear in the arena.</t>
         </is>
       </c>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="7" t="n"/>
     </row>
-    <row r="56" ht="21" customHeight="1">
-      <c r="A56" s="18" t="inlineStr">
+    <row r="56" ht="64" customHeight="1">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>N-10</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>Run more than 40 m out during a wave</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>the spiders do not follow. Clear wave 5 and the Queen -&gt; the scoreboard names a winner. Then type .nyar event disable spider-swarm so it does not repeat next week.</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n"/>
+    </row>
+    <row r="57" ht="21" customHeight="1">
+      <c r="A57" s="18" t="inlineStr">
         <is>
           <t>N-11 — Spider hunting grounds: spiders roam a whole region and hunt whoever is inside</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="49" customHeight="1">
-      <c r="A57" s="15" t="inlineStr">
+    <row r="58" ht="49" customHeight="1">
+      <c r="A58" s="15" t="inlineStr">
         <is>
           <t>N-11</t>
         </is>
       </c>
-      <c r="B57" s="15" t="n">
+      <c r="B58" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="C58" s="15" t="inlineStr">
         <is>
           <t>Type .nyar template use spider-hunting-grounds, .nyar event enable spider-hunting-grounds, .nyar event start spider-hunting-grounds.</t>
         </is>
       </c>
-      <c r="D57" s="15" t="inlineStr"/>
-      <c r="E57" s="7" t="n"/>
-      <c r="F57" s="7" t="n"/>
-    </row>
-    <row r="58" ht="19" customHeight="1">
-      <c r="A58" s="15" t="inlineStr">
-        <is>
-          <t>N-11</t>
-        </is>
-      </c>
-      <c r="B58" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C58" s="15" t="inlineStr">
-        <is>
-          <t>The player inside Dunley waits in the open</t>
-        </is>
-      </c>
-      <c r="D58" s="15" t="inlineStr">
-        <is>
-          <t>within a few minutes spider groups find them.</t>
-        </is>
-      </c>
+      <c r="D58" s="15" t="inlineStr"/>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="7" t="n"/>
     </row>
@@ -4630,16 +4642,16 @@
         </is>
       </c>
       <c r="B59" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>That player runs out of the region across the border</t>
+          <t>The player inside Dunley waits in the open</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>the spiders stop at the border and turn back.</t>
+          <t>within a few minutes spider groups find them.</t>
         </is>
       </c>
       <c r="E59" s="7" t="n"/>
@@ -4652,242 +4664,242 @@
         </is>
       </c>
       <c r="B60" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>The player outside the region stays outside</t>
+          <t>That player runs out of the region across the border</t>
         </is>
       </c>
       <c r="D60" s="15" t="inlineStr">
         <is>
-          <t>no spiders come for them.</t>
+          <t>the spiders stop at the border and turn back.</t>
         </is>
       </c>
       <c r="E60" s="7" t="n"/>
       <c r="F60" s="7" t="n"/>
     </row>
-    <row r="61" ht="34" customHeight="1">
+    <row r="61" ht="19" customHeight="1">
       <c r="A61" s="15" t="inlineStr">
         <is>
           <t>N-11</t>
         </is>
       </c>
       <c r="B61" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>Watch spiders approach from far away</t>
+          <t>The player outside the region stays outside</t>
         </is>
       </c>
       <c r="D61" s="15" t="inlineStr">
         <is>
-          <t>you never see one appear out of nowhere close to you.</t>
+          <t>no spiders come for them.</t>
         </is>
       </c>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="7" t="n"/>
     </row>
-    <row r="62" ht="21" customHeight="1">
-      <c r="A62" s="18" t="inlineStr">
+    <row r="62" ht="34" customHeight="1">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>N-11</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>Watch spiders approach from far away</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>you never see one appear out of nowhere close to you.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="7" t="n"/>
+    </row>
+    <row r="63" ht="21" customHeight="1">
+      <c r="A63" s="18" t="inlineStr">
         <is>
           <t>N-12 — A regional ambush: only players inside the region are picked</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="34" customHeight="1">
-      <c r="A63" s="15" t="inlineStr">
+    <row r="64" ht="34" customHeight="1">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>N-12</t>
         </is>
       </c>
-      <c r="B63" s="15" t="n">
+      <c r="B64" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C63" s="15" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
         <is>
           <t>Type .nyar template use graveyard-waves as farbane-ambush, then .nyar event enable farbane-ambush.</t>
         </is>
       </c>
-      <c r="D63" s="15" t="inlineStr"/>
-      <c r="E63" s="7" t="n"/>
-      <c r="F63" s="7" t="n"/>
-    </row>
-    <row r="64" ht="49" customHeight="1">
-      <c r="A64" s="15" t="inlineStr">
-        <is>
-          <t>N-12</t>
-        </is>
-      </c>
-      <c r="B64" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar event set farbane-ambush action.scope FarbaneWoods and .nyar event set farbane-ambush action.regionLock true</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="inlineStr">
-        <is>
-          <t>each confirms.</t>
-        </is>
-      </c>
+      <c r="D64" s="15" t="inlineStr"/>
       <c r="E64" s="7" t="n"/>
       <c r="F64" s="7" t="n"/>
     </row>
-    <row r="65" ht="34" customHeight="1">
+    <row r="65" ht="49" customHeight="1">
       <c r="A65" s="15" t="inlineStr">
         <is>
           <t>N-12</t>
         </is>
       </c>
       <c r="B65" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>With one player in Farbane Woods and one elsewhere, type .nyar event start farbane-ambush</t>
+          <t>Type .nyar event set farbane-ambush action.scope FarbaneWoods and .nyar event set farbane-ambush action.regionLock true</t>
         </is>
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>the skeletons appear only near the player in Farbane Woods.</t>
+          <t>each confirms.</t>
         </is>
       </c>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="7" t="n"/>
     </row>
-    <row r="66" ht="19" customHeight="1">
+    <row r="66" ht="34" customHeight="1">
       <c r="A66" s="15" t="inlineStr">
         <is>
           <t>N-12</t>
         </is>
       </c>
       <c r="B66" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>That player runs out of Farbane Woods</t>
+          <t>With one player in Farbane Woods and one elsewhere, type .nyar event start farbane-ambush</t>
         </is>
       </c>
       <c r="D66" s="15" t="inlineStr">
         <is>
-          <t>the skeletons do not follow across the border.</t>
+          <t>the skeletons appear only near the player in Farbane Woods.</t>
         </is>
       </c>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="7" t="n"/>
     </row>
-    <row r="67" ht="21" customHeight="1">
-      <c r="A67" s="18" t="inlineStr">
+    <row r="67" ht="19" customHeight="1">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>N-12</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>That player runs out of Farbane Woods</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>the skeletons do not follow across the border.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n"/>
+    </row>
+    <row r="68" ht="21" customHeight="1">
+      <c r="A68" s="18" t="inlineStr">
         <is>
           <t>N-13 — Bandit revenge: warnings, then a private hunt</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="34" customHeight="1">
-      <c r="A68" s="15" t="inlineStr">
+    <row r="69" ht="34" customHeight="1">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>N-13</t>
         </is>
       </c>
-      <c r="B68" s="15" t="n">
+      <c r="B69" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C69" s="15" t="inlineStr">
         <is>
           <t>Type .nyar template use bandit-revenge, .nyar event enable bandit-revenge.</t>
         </is>
       </c>
-      <c r="D68" s="15" t="inlineStr"/>
-      <c r="E68" s="7" t="n"/>
-      <c r="F68" s="7" t="n"/>
-    </row>
-    <row r="69" ht="64" customHeight="1">
-      <c r="A69" s="15" t="inlineStr">
-        <is>
-          <t>N-13</t>
-        </is>
-      </c>
-      <c r="B69" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C69" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar event set bandit-revenge trigger.warnAt 4,8 first, then .nyar event set bandit-revenge trigger.heat 12 (a small-server setting; the warnings must stay below the heat, so this order)</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr">
-        <is>
-          <t>each confirms.</t>
-        </is>
-      </c>
+      <c r="D69" s="15" t="inlineStr"/>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="7" t="n"/>
     </row>
-    <row r="70" ht="34" customHeight="1">
+    <row r="70" ht="64" customHeight="1">
       <c r="A70" s="15" t="inlineStr">
         <is>
           <t>N-13</t>
         </is>
       </c>
       <c r="B70" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Kill bandits</t>
+          <t>Type .nyar event set bandit-revenge trigger.warnAt 4,8 first, then .nyar event set bandit-revenge trigger.heat 12 (a small-server setting; the warnings must stay below the heat, so this order)</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>after 4 and after 8 kills you get a private warning; the other player sees nothing.</t>
+          <t>each confirms.</t>
         </is>
       </c>
       <c r="E70" s="7" t="n"/>
       <c r="F70" s="7" t="n"/>
     </row>
-    <row r="71" ht="49" customHeight="1">
+    <row r="71" ht="34" customHeight="1">
       <c r="A71" s="15" t="inlineStr">
         <is>
           <t>N-13</t>
         </is>
       </c>
       <c r="B71" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>Kill 12</t>
+          <t>Kill bandits</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>everyone sees an alert that names no one; you get a private line; bandits appear 20-40 m from you and hunt you.</t>
+          <t>after 4 and after 8 kills you get a private warning; the other player sees nothing.</t>
         </is>
       </c>
       <c r="E71" s="7" t="n"/>
       <c r="F71" s="7" t="n"/>
     </row>
-    <row r="72" ht="19" customHeight="1">
+    <row r="72" ht="49" customHeight="1">
       <c r="A72" s="15" t="inlineStr">
         <is>
           <t>N-13</t>
         </is>
       </c>
       <c r="B72" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>The second player stands near you</t>
+          <t>Kill 12</t>
         </is>
       </c>
       <c r="D72" s="15" t="inlineStr">
         <is>
-          <t>the bandits keep going after you, not them.</t>
+          <t>everyone sees an alert that names no one; you get a private line; bandits appear 20-40 m from you and hunt you.</t>
         </is>
       </c>
       <c r="E72" s="7" t="n"/>
@@ -4900,107 +4912,107 @@
         </is>
       </c>
       <c r="B73" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Clear all three waves</t>
+          <t>The second player stands near you</t>
         </is>
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>you get a private end line.</t>
+          <t>the bandits keep going after you, not them.</t>
         </is>
       </c>
       <c r="E73" s="7" t="n"/>
       <c r="F73" s="7" t="n"/>
     </row>
-    <row r="74" ht="21" customHeight="1">
-      <c r="A74" s="18" t="inlineStr">
+    <row r="74" ht="19" customHeight="1">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>N-13</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>Clear all three waves</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>you get a private end line.</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="n"/>
+      <c r="F74" s="7" t="n"/>
+    </row>
+    <row r="75" ht="21" customHeight="1">
+      <c r="A75" s="18" t="inlineStr">
         <is>
           <t>N-14 — Zombie apocalypse: a two-hour outbreak the server has to survive</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="49" customHeight="1">
-      <c r="A75" s="15" t="inlineStr">
+    <row r="76" ht="34" customHeight="1">
+      <c r="A76" s="15" t="inlineStr">
         <is>
           <t>N-14</t>
         </is>
       </c>
-      <c r="B75" s="15" t="n">
+      <c r="B76" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C75" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar template use zombie-apocalypse, .nyar event enable zombie-apocalypse, and .nyar event set zombie-apocalypse durationSeconds 7200.</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr"/>
-      <c r="E75" s="7" t="n"/>
-      <c r="F75" s="7" t="n"/>
-    </row>
-    <row r="76" ht="49" customHeight="1">
-      <c r="A76" s="15" t="inlineStr">
-        <is>
-          <t>N-14</t>
-        </is>
-      </c>
-      <c r="B76" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Standing at the spot to defend, type .nyar event start zombie-apocalypse</t>
-        </is>
-      </c>
-      <c r="D76" s="15" t="inlineStr">
-        <is>
-          <t>chat says the dead rise; .nyar event info zombie-apocalypse lists three hotspots with their regions.</t>
-        </is>
-      </c>
+          <t>Type .nyar template use zombie-apocalypse and .nyar event set zombie-apocalypse durationSeconds 7200.</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr"/>
       <c r="E76" s="7" t="n"/>
       <c r="F76" s="7" t="n"/>
     </row>
-    <row r="77" ht="34" customHeight="1">
+    <row r="77" ht="64" customHeight="1">
       <c r="A77" s="15" t="inlineStr">
         <is>
           <t>N-14</t>
         </is>
       </c>
       <c r="B77" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Players spread out over the map</t>
+          <t>Walk to the place to defend and type .nyar event set zombie-apocalypse action.goal here, then .nyar event set zombie-apocalypse action.goal.name Crossroads, then .nyar event enable zombie-apocalypse</t>
         </is>
       </c>
       <c r="D77" s="15" t="inlineStr">
         <is>
-          <t>within a few minutes roamers find players far from the defended spot.</t>
+          <t>each confirms.</t>
         </is>
       </c>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="7" t="n"/>
     </row>
-    <row r="78" ht="34" customHeight="1">
+    <row r="78" ht="49" customHeight="1">
       <c r="A78" s="15" t="inlineStr">
         <is>
           <t>N-14</t>
         </is>
       </c>
       <c r="B78" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>After 10 minutes, then every 30</t>
+          <t>When everyone is ready, type .nyar event start zombie-apocalypse from anywhere</t>
         </is>
       </c>
       <c r="D78" s="15" t="inlineStr">
         <is>
-          <t>chat announces each horde rising and its march at each quarter.</t>
+          <t>chat says the dead rise; .nyar event info zombie-apocalypse lists three hotspots and the defended place.</t>
         </is>
       </c>
       <c r="E78" s="7" t="n"/>
@@ -5013,16 +5025,16 @@
         </is>
       </c>
       <c r="B79" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>Stand in a horde's path</t>
+          <t>Players spread out over the map</t>
         </is>
       </c>
       <c r="D79" s="15" t="inlineStr">
         <is>
-          <t>it stops to fight while you hold within about 60 m of its front.</t>
+          <t>within a few minutes roamers find players far from the defended place.</t>
         </is>
       </c>
       <c r="E79" s="7" t="n"/>
@@ -5035,58 +5047,62 @@
         </is>
       </c>
       <c r="B80" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Play it out</t>
+          <t>After 10 minutes, then every 30</t>
         </is>
       </c>
       <c r="D80" s="15" t="inlineStr">
         <is>
-          <t>chat shows the outcome (won, lost or survived) and the scoreboard.</t>
+          <t>chat announces each horde rising and its march towards the place.</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="7" t="n"/>
     </row>
-    <row r="81" ht="21" customHeight="1">
-      <c r="A81" s="18" t="inlineStr">
+    <row r="81" ht="49" customHeight="1">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>N-14</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>Hold the place, or stand in a horde's path</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>it stops to fight while you hold within about 60 m of it. Play it out -&gt; chat shows the outcome (won, lost or survived) and the scoreboard.</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="n"/>
+      <c r="F81" s="7" t="n"/>
+    </row>
+    <row r="82" ht="21" customHeight="1">
+      <c r="A82" s="18" t="inlineStr">
         <is>
           <t>N-15 — A monster that cannot reach you is moved, and a wave never hangs</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="49" customHeight="1">
-      <c r="A82" s="15" t="inlineStr">
+    <row r="83" ht="49" customHeight="1">
+      <c r="A83" s="15" t="inlineStr">
         <is>
           <t>N-15</t>
         </is>
       </c>
-      <c r="B82" s="15" t="n">
+      <c r="B83" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C82" s="15" t="inlineStr">
+      <c r="C83" s="15" t="inlineStr">
         <is>
           <t>Stand at the foot of the rock. Type .nyar template use spider-swarm as stuck-test, .nyar event enable stuck-test, .nyar event start stuck-test.</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr"/>
-      <c r="E82" s="7" t="n"/>
-      <c r="F82" s="7" t="n"/>
-    </row>
-    <row r="83" ht="34" customHeight="1">
-      <c r="A83" s="15" t="inlineStr">
-        <is>
-          <t>N-15</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C83" s="15" t="inlineStr">
-        <is>
-          <t>As soon as spiders appear, climb onto the rock and stay within about 20 m of them without attacking.</t>
         </is>
       </c>
       <c r="D83" s="15" t="inlineStr"/>
@@ -5100,18 +5116,14 @@
         </is>
       </c>
       <c r="B84" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Wait about 2 minutes</t>
-        </is>
-      </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>type .nyar event info stuck-test: the unit watch line reads 'stuck now' above 0.</t>
-        </is>
-      </c>
+          <t>As soon as spiders appear, climb onto the rock and stay within about 20 m of them without attacking.</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr"/>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="7" t="n"/>
     </row>
@@ -5122,352 +5134,352 @@
         </is>
       </c>
       <c r="B85" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>Walk 150 m away for a minute, then come back</t>
+          <t>Wait about 2 minutes</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
         <is>
-          <t>the stuck spiders are no longer at the foot of the rock.</t>
+          <t>type .nyar event info stuck-test: the unit watch line reads 'stuck now' above 0.</t>
         </is>
       </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="7" t="n"/>
     </row>
-    <row r="86" ht="19" customHeight="1">
+    <row r="86" ht="34" customHeight="1">
       <c r="A86" s="15" t="inlineStr">
         <is>
           <t>N-15</t>
         </is>
       </c>
       <c r="B86" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>While watching any spider</t>
+          <t>Walk 150 m away for a minute, then come back</t>
         </is>
       </c>
       <c r="D86" s="15" t="inlineStr">
         <is>
-          <t>none vanishes or appears in front of you.</t>
+          <t>the stuck spiders are no longer at the foot of the rock.</t>
         </is>
       </c>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="7" t="n"/>
     </row>
-    <row r="87" ht="21" customHeight="1">
-      <c r="A87" s="18" t="inlineStr">
+    <row r="87" ht="19" customHeight="1">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>N-15</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>While watching any spider</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>none vanishes or appears in front of you.</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n"/>
+      <c r="F87" s="7" t="n"/>
+    </row>
+    <row r="88" ht="21" customHeight="1">
+      <c r="A88" s="18" t="inlineStr">
         <is>
           <t>N-16 — Castles stay safe: no spawns or jumps inside claimed territory</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="34" customHeight="1">
-      <c r="A88" s="15" t="inlineStr">
+    <row r="89" ht="49" customHeight="1">
+      <c r="A89" s="15" t="inlineStr">
         <is>
           <t>N-16</t>
         </is>
       </c>
-      <c r="B88" s="15" t="n">
+      <c r="B89" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C88" s="15" t="inlineStr">
-        <is>
-          <t>Stand inside your castle territory. Type .nyar event start bandit-ambush (set up in N-05)</t>
-        </is>
-      </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>no bandits appear inside the territory.</t>
-        </is>
-      </c>
-      <c r="E88" s="7" t="n"/>
-      <c r="F88" s="7" t="n"/>
-    </row>
-    <row r="89" ht="34" customHeight="1">
-      <c r="A89" s="15" t="inlineStr">
-        <is>
-          <t>N-16</t>
-        </is>
-      </c>
-      <c r="B89" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="C89" s="15" t="inlineStr">
         <is>
-          <t>Start roaming-hunters (N-07) while one player is in their castle and one outside</t>
+          <t>Stand inside your castle territory with nobody else online outside one. Type .nyar event start graveyard-waves (set up in N-06)</t>
         </is>
       </c>
       <c r="D89" s="15" t="inlineStr">
         <is>
-          <t>only the outside player gets a squad.</t>
+          <t>no skeletons come for you: a player in their castle is never picked.</t>
         </is>
       </c>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="7" t="n"/>
     </row>
-    <row r="90" ht="19" customHeight="1">
+    <row r="90" ht="34" customHeight="1">
       <c r="A90" s="15" t="inlineStr">
         <is>
           <t>N-16</t>
         </is>
       </c>
       <c r="B90" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>During the apocalypse (N-14), shelter in the castle</t>
+          <t>Start roaming-hunters (N-07) while one player is in their castle and one outside</t>
         </is>
       </c>
       <c r="D90" s="15" t="inlineStr">
         <is>
-          <t>roamers do not appear inside it.</t>
+          <t>only the outside player gets a squad.</t>
         </is>
       </c>
       <c r="E90" s="7" t="n"/>
       <c r="F90" s="7" t="n"/>
     </row>
-    <row r="91" ht="21" customHeight="1">
-      <c r="A91" s="18" t="inlineStr">
+    <row r="91" ht="19" customHeight="1">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>N-16</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C91" s="15" t="inlineStr">
+        <is>
+          <t>During the apocalypse (N-14), shelter in the castle</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>roamers do not appear inside it.</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="n"/>
+      <c r="F91" s="7" t="n"/>
+    </row>
+    <row r="92" ht="21" customHeight="1">
+      <c r="A92" s="18" t="inlineStr">
         <is>
           <t>N-17 — Stopping things: event stop, switching a kind off, and the emergency stop</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="49" customHeight="1">
-      <c r="A92" s="15" t="inlineStr">
+    <row r="93" ht="49" customHeight="1">
+      <c r="A93" s="15" t="inlineStr">
         <is>
           <t>N-17</t>
         </is>
       </c>
-      <c r="B92" s="15" t="n">
+      <c r="B93" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C92" s="15" t="inlineStr">
+      <c r="C93" s="15" t="inlineStr">
         <is>
           <t>Start graveyard-waves, then type .nyar event stop graveyard-waves</t>
         </is>
       </c>
-      <c r="D92" s="15" t="inlineStr">
+      <c r="D93" s="15" t="inlineStr">
         <is>
           <t>the scoreboard shows; the skeletons disappear within about a minute; .nyar status reads 'tracked units: 0'.</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="n"/>
-      <c r="F92" s="7" t="n"/>
-    </row>
-    <row r="93" ht="19" customHeight="1">
-      <c r="A93" s="15" t="inlineStr">
-        <is>
-          <t>N-17</t>
-        </is>
-      </c>
-      <c r="B93" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C93" s="15" t="inlineStr">
-        <is>
-          <t>Start bandit-ambush, then type .nyar pillar spawns off</t>
-        </is>
-      </c>
-      <c r="D93" s="15" t="inlineStr">
-        <is>
-          <t>the ambush ends and its bandits disappear.</t>
         </is>
       </c>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="7" t="n"/>
     </row>
-    <row r="94" ht="34" customHeight="1">
+    <row r="94" ht="19" customHeight="1">
       <c r="A94" s="15" t="inlineStr">
         <is>
           <t>N-17</t>
         </is>
       </c>
       <c r="B94" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar pillar spawns on, start two spawn events, then type .nyar purge and .nyar purge confirm</t>
+          <t>Start bandit-ambush, then type .nyar pillar spawns off</t>
         </is>
       </c>
       <c r="D94" s="15" t="inlineStr">
         <is>
-          <t>everything ends and every spawned monster is gone within a minute; nothing is shown in chat.</t>
+          <t>the ambush ends and its bandits disappear.</t>
         </is>
       </c>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="7" t="n"/>
     </row>
-    <row r="95" ht="19" customHeight="1">
+    <row r="95" ht="34" customHeight="1">
       <c r="A95" s="15" t="inlineStr">
         <is>
           <t>N-17</t>
         </is>
       </c>
       <c r="B95" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C95" s="15" t="inlineStr">
         <is>
-          <t>Try .nyar event start bandit-ambush right after</t>
+          <t>Type .nyar pillar spawns on, start two spawn events, then type .nyar purge and .nyar purge confirm</t>
         </is>
       </c>
       <c r="D95" s="15" t="inlineStr">
         <is>
-          <t>it is refused for about 4 minutes.</t>
+          <t>everything ends and every spawned monster is gone within a minute; nothing is shown in chat.</t>
         </is>
       </c>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="7" t="n"/>
     </row>
-    <row r="96" ht="21" customHeight="1">
-      <c r="A96" s="18" t="inlineStr">
-        <is>
-          <t>N-18 — Timed waves: the next wave comes whether you are ready or not</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="34" customHeight="1">
-      <c r="A97" s="15" t="inlineStr">
+    <row r="96" ht="19" customHeight="1">
+      <c r="A96" s="15" t="inlineStr">
+        <is>
+          <t>N-17</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C96" s="15" t="inlineStr">
+        <is>
+          <t>Try .nyar event start bandit-ambush right after</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>it is refused for about 4 minutes.</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="n"/>
+      <c r="F96" s="7" t="n"/>
+    </row>
+    <row r="97" ht="21" customHeight="1">
+      <c r="A97" s="18" t="inlineStr">
+        <is>
+          <t>N-18 — Timed waves at a muster point: the next wave comes whether you are ready or not</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="49" customHeight="1">
+      <c r="A98" s="15" t="inlineStr">
         <is>
           <t>N-18</t>
         </is>
       </c>
-      <c r="B97" s="15" t="n">
+      <c r="B98" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C97" s="15" t="inlineStr">
-        <is>
-          <t>Type .nyar template use militia-muster-timed, .nyar event enable militia-muster-timed.</t>
-        </is>
-      </c>
-      <c r="D97" s="15" t="inlineStr"/>
-      <c r="E97" s="7" t="n"/>
-      <c r="F97" s="7" t="n"/>
-    </row>
-    <row r="98" ht="34" customHeight="1">
-      <c r="A98" s="15" t="inlineStr">
-        <is>
-          <t>N-18</t>
-        </is>
-      </c>
-      <c r="B98" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Stand in open ground and type .nyar event start militia-muster-timed</t>
+          <t>Type .nyar template use militia-muster-timed. At an open spot in Dunley Farmlands type .nyar event set militia-muster-timed location here</t>
         </is>
       </c>
       <c r="D98" s="15" t="inlineStr">
         <is>
-          <t>wave 1 (6 militia) appears around you.</t>
+          <t>it confirms.</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="7" t="n"/>
     </row>
-    <row r="99" ht="34" customHeight="1">
+    <row r="99" ht="49" customHeight="1">
       <c r="A99" s="15" t="inlineStr">
         <is>
           <t>N-18</t>
         </is>
       </c>
       <c r="B99" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>Do not fight for a while</t>
-        </is>
-      </c>
-      <c r="D99" s="15" t="inlineStr">
-        <is>
-          <t>about 75 seconds after the start, wave 2 (9 militia) arrives while wave 1 is still alive.</t>
-        </is>
-      </c>
+          <t>Give it a time limit: .nyar event set militia-muster-timed durationSeconds 900 (15 minutes), then .nyar event enable militia-muster-timed.</t>
+        </is>
+      </c>
+      <c r="D99" s="15" t="inlineStr"/>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="7" t="n"/>
     </row>
-    <row r="100" ht="49" customHeight="1">
+    <row r="100" ht="34" customHeight="1">
       <c r="A100" s="15" t="inlineStr">
         <is>
           <t>N-18</t>
         </is>
       </c>
       <c r="B100" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Fight the rest</t>
+          <t>With the players at the spot, type .nyar event start militia-muster-timed</t>
         </is>
       </c>
       <c r="D100" s="15" t="inlineStr">
         <is>
-          <t>waves keep coming every 75 seconds; wave 5 brings the militia leader; the scoreboard names a winner at the end.</t>
+          <t>wave 1 (6 militia) appears there.</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="7" t="n"/>
     </row>
-    <row r="101" ht="21" customHeight="1">
-      <c r="A101" s="18" t="inlineStr">
-        <is>
-          <t>N-19 — Onslaught: random waves, surprise bosses, and no running away</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="49" customHeight="1">
+    <row r="101" ht="34" customHeight="1">
+      <c r="A101" s="15" t="inlineStr">
+        <is>
+          <t>N-18</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t>Hold back</t>
+        </is>
+      </c>
+      <c r="D101" s="15" t="inlineStr">
+        <is>
+          <t>about 75 seconds after the start, wave 2 (9 militia) arrives while wave 1 is still alive.</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n"/>
+      <c r="F101" s="7" t="n"/>
+    </row>
+    <row r="102" ht="64" customHeight="1">
       <c r="A102" s="15" t="inlineStr">
         <is>
-          <t>N-19</t>
+          <t>N-18</t>
         </is>
       </c>
       <c r="B102" s="15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar template use undead-onslaught, .nyar event enable undead-onslaught, then .nyar event start undead-onslaught in open ground</t>
+          <t>Fight on</t>
         </is>
       </c>
       <c r="D102" s="15" t="inlineStr">
         <is>
-          <t>about 12 undead appear around you.</t>
+          <t>a new wave every 75 seconds; wave 5 brings the militia leader; the scoreboard names a winner. If you are still fighting at 15 minutes, the event ends.</t>
         </is>
       </c>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="7" t="n"/>
     </row>
-    <row r="103" ht="34" customHeight="1">
-      <c r="A103" s="15" t="inlineStr">
-        <is>
-          <t>N-19</t>
-        </is>
-      </c>
-      <c r="B103" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C103" s="15" t="inlineStr">
-        <is>
-          <t>Clear wave 1 or wait 75 seconds</t>
-        </is>
-      </c>
-      <c r="D103" s="15" t="inlineStr">
-        <is>
-          <t>wave 2 brings different undead and one V Blood boss.</t>
-        </is>
-      </c>
-      <c r="E103" s="7" t="n"/>
-      <c r="F103" s="7" t="n"/>
+    <row r="103" ht="21" customHeight="1">
+      <c r="A103" s="18" t="inlineStr">
+        <is>
+          <t>N-19 — Onslaught: random waves, surprise bosses, and no running away</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="49" customHeight="1">
       <c r="A104" s="15" t="inlineStr">
@@ -5476,38 +5488,34 @@
         </is>
       </c>
       <c r="B104" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C104" s="15" t="inlineStr">
         <is>
-          <t>Both players run more than 60 m away and wait</t>
-        </is>
-      </c>
-      <c r="D104" s="15" t="inlineStr">
-        <is>
-          <t>about a minute later the undead come after the nearest of you, arriving near you rather than on top of you.</t>
-        </is>
-      </c>
+          <t>Type .nyar template use undead-onslaught. At an open spot near a graveyard type .nyar event set undead-onslaught location here.</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr"/>
       <c r="E104" s="7" t="n"/>
       <c r="F104" s="7" t="n"/>
     </row>
-    <row r="105" ht="19" customHeight="1">
+    <row r="105" ht="64" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
         <is>
           <t>N-19</t>
         </is>
       </c>
       <c r="B105" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C105" s="15" t="inlineStr">
         <is>
-          <t>Go into your castle's territory</t>
+          <t>Set how long they wait before giving chase: .nyar event set undead-onslaught action.pursuit 90, then .nyar event enable undead-onslaught and .nyar event start undead-onslaught</t>
         </is>
       </c>
       <c r="D105" s="15" t="inlineStr">
         <is>
-          <t>they do not follow you in.</t>
+          <t>about 12 undead appear at the spot.</t>
         </is>
       </c>
       <c r="E105" s="7" t="n"/>
@@ -5520,67 +5528,71 @@
         </is>
       </c>
       <c r="B106" s="15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C106" s="15" t="inlineStr">
         <is>
-          <t>Stop it (.nyar event stop undead-onslaught) and start it again</t>
+          <t>Clear wave 1 or wait 75 seconds</t>
         </is>
       </c>
       <c r="D106" s="15" t="inlineStr">
         <is>
-          <t>the waves and bosses are different.</t>
+          <t>wave 2 brings different undead and one V Blood boss.</t>
         </is>
       </c>
       <c r="E106" s="7" t="n"/>
       <c r="F106" s="7" t="n"/>
     </row>
-    <row r="107" ht="21" customHeight="1">
-      <c r="A107" s="18" t="inlineStr">
-        <is>
-          <t>E-01 — Build your own event from chat, the way a new admin would</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="19" customHeight="1">
+    <row r="107" ht="64" customHeight="1">
+      <c r="A107" s="15" t="inlineStr">
+        <is>
+          <t>N-19</t>
+        </is>
+      </c>
+      <c r="B107" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C107" s="15" t="inlineStr">
+        <is>
+          <t>Both players run more than 60 m away and wait</t>
+        </is>
+      </c>
+      <c r="D107" s="15" t="inlineStr">
+        <is>
+          <t>about 90 seconds later the undead come after the nearest of you, arriving near you rather than on top of you. Go into your castle's territory -&gt; they do not follow you in.</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="n"/>
+      <c r="F107" s="7" t="n"/>
+    </row>
+    <row r="108" ht="34" customHeight="1">
       <c r="A108" s="15" t="inlineStr">
         <is>
-          <t>E-01</t>
+          <t>N-19</t>
         </is>
       </c>
       <c r="B108" s="15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C108" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event new my-event spawns</t>
+          <t>Stop it (.nyar event stop undead-onslaught) and start it again</t>
         </is>
       </c>
       <c r="D108" s="15" t="inlineStr">
         <is>
-          <t>a switched-off event is created.</t>
+          <t>the waves and bosses are different.</t>
         </is>
       </c>
       <c r="E108" s="7" t="n"/>
       <c r="F108" s="7" t="n"/>
     </row>
-    <row r="109" ht="49" customHeight="1">
-      <c r="A109" s="15" t="inlineStr">
-        <is>
-          <t>E-01</t>
-        </is>
-      </c>
-      <c r="B109" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C109" s="15" t="inlineStr">
-        <is>
-          <t>Use .nyar event set my-event ... to choose units (action.units, e.g. CHAR_Forest_Wolf:4), waves, the location (location here) and a level (action.modifiers.level 30).</t>
-        </is>
-      </c>
-      <c r="D109" s="15" t="inlineStr"/>
-      <c r="E109" s="7" t="n"/>
-      <c r="F109" s="7" t="n"/>
+    <row r="109" ht="21" customHeight="1">
+      <c r="A109" s="18" t="inlineStr">
+        <is>
+          <t>E-01 — Build your own event from chat, the way a new admin would</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="19" customHeight="1">
       <c r="A110" s="15" t="inlineStr">
@@ -5589,160 +5601,200 @@
         </is>
       </c>
       <c r="B110" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C110" s="15" t="inlineStr">
         <is>
-          <t>Type .nyar event info my-event, then enable and start it</t>
+          <t>Type .nyar event new my-event spawns</t>
         </is>
       </c>
       <c r="D110" s="15" t="inlineStr">
         <is>
-          <t>it runs as you set it.</t>
+          <t>a switched-off event is created.</t>
         </is>
       </c>
       <c r="E110" s="7" t="n"/>
       <c r="F110" s="7" t="n"/>
     </row>
-    <row r="111" ht="19" customHeight="1">
+    <row r="111" ht="49" customHeight="1">
       <c r="A111" s="15" t="inlineStr">
         <is>
           <t>E-01</t>
         </is>
       </c>
       <c r="B111" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C111" s="15" t="inlineStr">
         <is>
-          <t>Note every reply that confused you, word for word.</t>
+          <t>Use .nyar event set my-event ... to choose units (action.units, e.g. CHAR_Forest_Wolf:4), waves, the location (location here) and a level (action.modifiers.level 30).</t>
         </is>
       </c>
       <c r="D111" s="15" t="inlineStr"/>
       <c r="E111" s="7" t="n"/>
       <c r="F111" s="7" t="n"/>
     </row>
-    <row r="112" ht="21" customHeight="1">
-      <c r="A112" s="18" t="inlineStr">
-        <is>
-          <t>E-02 — A second player joins someone else's fight</t>
-        </is>
-      </c>
+    <row r="112" ht="19" customHeight="1">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t>E-01</t>
+        </is>
+      </c>
+      <c r="B112" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C112" s="15" t="inlineStr">
+        <is>
+          <t>Type .nyar event info my-event, then enable and start it</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="inlineStr">
+        <is>
+          <t>it runs as you set it.</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="n"/>
+      <c r="F112" s="7" t="n"/>
     </row>
     <row r="113" ht="19" customHeight="1">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-01</t>
         </is>
       </c>
       <c r="B113" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C113" s="15" t="inlineStr">
         <is>
-          <t>Player one triggers N-08 or N-13</t>
-        </is>
-      </c>
-      <c r="D113" s="15" t="inlineStr">
-        <is>
-          <t>monsters hunt player one.</t>
-        </is>
-      </c>
+          <t>Note every reply that confused you, word for word.</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr"/>
       <c r="E113" s="7" t="n"/>
       <c r="F113" s="7" t="n"/>
     </row>
-    <row r="114" ht="19" customHeight="1">
-      <c r="A114" s="15" t="inlineStr">
+    <row r="114" ht="21" customHeight="1">
+      <c r="A114" s="18" t="inlineStr">
+        <is>
+          <t>E-02 — A second player joins someone else's fight</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="19" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
         <is>
           <t>E-02</t>
         </is>
       </c>
-      <c r="B114" s="15" t="n">
+      <c r="B115" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C115" s="15" t="inlineStr">
+        <is>
+          <t>Player one triggers N-08 or N-13</t>
+        </is>
+      </c>
+      <c r="D115" s="15" t="inlineStr">
+        <is>
+          <t>monsters hunt player one.</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="n"/>
+      <c r="F115" s="7" t="n"/>
+    </row>
+    <row r="116" ht="19" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>E-02</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="C114" s="15" t="inlineStr">
+      <c r="C116" s="15" t="inlineStr">
         <is>
           <t>Player two joins the fight and attacks the monsters</t>
         </is>
       </c>
-      <c r="D114" s="15" t="inlineStr">
+      <c r="D116" s="15" t="inlineStr">
         <is>
           <t>note who they turn on, and who gets kill credit.</t>
         </is>
       </c>
-      <c r="E114" s="7" t="n"/>
-      <c r="F114" s="7" t="n"/>
-    </row>
-    <row r="115" ht="21" customHeight="1">
-      <c r="A115" s="18" t="inlineStr">
-        <is>
-          <t>C-01 — Measurement: how the server feels during the busiest event</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="49" customHeight="1">
-      <c r="A116" s="15" t="inlineStr">
-        <is>
-          <t>C-01</t>
-        </is>
-      </c>
-      <c r="B116" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C116" s="15" t="inlineStr">
-        <is>
-          <t>At the start, at each horde rise and at the end, note how responsive the game feels (fine, slight lag, bad lag) and the time.</t>
-        </is>
-      </c>
-      <c r="D116" s="15" t="inlineStr"/>
       <c r="E116" s="7" t="n"/>
       <c r="F116" s="7" t="n"/>
     </row>
-    <row r="117" ht="34" customHeight="1">
-      <c r="A117" s="15" t="inlineStr">
+    <row r="117" ht="21" customHeight="1">
+      <c r="A117" s="18" t="inlineStr">
+        <is>
+          <t>C-01 — Measurement: how the server feels during the busiest event</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="49" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
         <is>
           <t>C-01</t>
         </is>
       </c>
-      <c r="B117" s="15" t="n">
+      <c r="B118" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C118" s="15" t="inlineStr">
+        <is>
+          <t>At the start, at each horde rise and at the end, note how responsive the game feels (fine, slight lag, bad lag) and the time.</t>
+        </is>
+      </c>
+      <c r="D118" s="15" t="inlineStr"/>
+      <c r="E118" s="7" t="n"/>
+      <c r="F118" s="7" t="n"/>
+    </row>
+    <row r="119" ht="34" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>C-01</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="C117" s="15" t="inlineStr">
+      <c r="C119" s="15" t="inlineStr">
         <is>
           <t>If something felt bad, write what you were doing and how many monsters were around.</t>
         </is>
       </c>
-      <c r="D117" s="15" t="inlineStr"/>
-      <c r="E117" s="7" t="n"/>
-      <c r="F117" s="7" t="n"/>
+      <c r="D119" s="15" t="inlineStr"/>
+      <c r="E119" s="7" t="n"/>
+      <c r="F119" s="7" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F117"/>
+  <autoFilter ref="A1:F119"/>
   <mergeCells count="22">
-    <mergeCell ref="A74:F74"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A101:F101"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="A57:F57"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="A96:F96"/>
-    <mergeCell ref="A91:F91"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A81:F81"/>
-    <mergeCell ref="A115:F115"/>
-    <mergeCell ref="A112:F112"/>
+    <mergeCell ref="A97:F97"/>
+    <mergeCell ref="A109:F109"/>
+    <mergeCell ref="A63:F63"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A67:F67"/>
-    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A117:F117"/>
+    <mergeCell ref="A92:F92"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A114:F114"/>
     <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A107:F107"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="A88:F88"/>
     <mergeCell ref="A7:F7"/>
   </mergeCells>
-  <conditionalFormatting sqref="E2:E117">
+  <conditionalFormatting sqref="E2:E119">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>E2="OK"</formula>
     </cfRule>
@@ -5754,7 +5806,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Problem,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6267,7 +6319,7 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIF('Test steps'!$E$2:$E$117,"OK")</f>
+        <f>COUNTIF('Test steps'!$E$2:$E$119,"OK")</f>
         <v/>
       </c>
     </row>
@@ -6278,7 +6330,7 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIF('Test steps'!$E$2:$E$117,"Problem")</f>
+        <f>COUNTIF('Test steps'!$E$2:$E$119,"Problem")</f>
         <v/>
       </c>
     </row>
@@ -6289,7 +6341,7 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Test steps'!$E$2:$E$117,"Skipped")</f>
+        <f>COUNTIF('Test steps'!$E$2:$E$119,"Skipped")</f>
         <v/>
       </c>
     </row>

</xml_diff>